<commit_message>
feat(web): bundle JSZip library into HTML for 100% offline single-file usage
</commit_message>
<xml_diff>
--- a/moban.xlsx
+++ b/moban.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\systemdata\Documents\IPV6\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC781262-7968-48BF-BC53-C6CDADB83871}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{447BEED3-1AE7-4CE3-9177-67E618549470}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{3A5D6A27-01DA-4C4B-9259-5DA9547EE256}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="26">
   <si>
     <t>/</t>
   </si>
@@ -130,6 +130,14 @@
   <si>
     <t>从【2001:4860:4860::8800】
 到【2001:4860:4860::88ff】</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>IPv6地址数量</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>显示地址数量</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -619,7 +627,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B43EABC-031E-4A80-9AA0-A25C094EC4A3}">
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18.75" customWidth="1"/>
@@ -693,48 +701,46 @@
       </c>
     </row>
     <row r="7" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="8" t="s">
+      <c r="A7" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="B7" s="8"/>
+      <c r="C7" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D7" s="5"/>
+    </row>
+    <row r="8" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="B7" s="8"/>
-      <c r="C7" s="5"/>
-      <c r="D7" s="4"/>
-    </row>
-    <row r="8" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="2" t="s">
+      <c r="B8" s="8"/>
+      <c r="C8" s="5"/>
+      <c r="D8" s="4"/>
+    </row>
+    <row r="9" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B9" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="C9" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D9" s="7" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B9" s="1">
-        <v>0</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="D9" s="1"/>
     </row>
     <row r="10" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B10" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D10" s="1"/>
     </row>
@@ -743,10 +749,10 @@
         <v>0</v>
       </c>
       <c r="B11" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D11" s="1"/>
     </row>
@@ -755,22 +761,35 @@
         <v>0</v>
       </c>
       <c r="B12" s="1">
+        <v>2</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D12" s="1"/>
+    </row>
+    <row r="13" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B13" s="1">
         <v>3</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="C13" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="D12" s="1"/>
+      <c r="D13" s="1"/>
     </row>
   </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="A7:B7"/>
+  <mergeCells count="8">
+    <mergeCell ref="A8:B8"/>
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="A6:B6"/>
+    <mergeCell ref="A7:B7"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
update: sync excel export with new template v1.2.5
</commit_message>
<xml_diff>
--- a/moban.xlsx
+++ b/moban.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\systemdata\Documents\IPV6\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{447BEED3-1AE7-4CE3-9177-67E618549470}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB4CF67D-20AD-4016-AE40-8B8773414120}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{3A5D6A27-01DA-4C4B-9259-5DA9547EE256}"/>
   </bookViews>
@@ -133,11 +133,11 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>IPv6地址数量</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>显示地址数量</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>当前子网IPv6地址数量</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -702,11 +702,11 @@
     </row>
     <row r="7" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="9" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B7" s="8"/>
       <c r="C7" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D7" s="5"/>
     </row>

</xml_diff>